<commit_message>
Rewrite Sugar News 2026-08-31
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-31.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-31.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,156 +505,139 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="159.3" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>CEPEA统计显示，8月25日至29日圣保罗州糖厂含税水合乙醇均价为2.2020雷亚尔/升、较7月上涨3.11%，无水乙醇均价为2.4750雷亚尔/升、上涨1.59%，这是2026/27榨季圣保罗糖厂乙醇价格首次录得月度上涨。乙醇价格回升提高糖厂制醇收益，同时9月中南部降雨预报会压缩压榨窗口，糖厂增加乙醇生产或放慢压榨时会减少短期食糖产出。来源：UOL/Reuters（https://economia.uol.com.br/noticias/reuters/2026/08/31/cepea-registra-1-alta-mensal-no-preco-do-etanol-na-safra-202627-nas-usinas-de-sp.htm）。影响：利多糖价</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>利多：巴西圣保罗乙醇价格上涨提高制醇回报，并且降雨压缩压榨窗口会减少短期制糖用蔗和食糖产出，从而支撑原糖价格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="180" customHeight="1" s="2">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>ICE原糖期货8月31日收涨0.25美分至17.81美分/磅，8月累计上涨21.5%；Archer Consulting指出，巴西生物燃料价格恢复可能使糖厂暂时维持较高乙醇产量。乙醇收益改善会提高甘蔗流向燃料乙醇的吸引力，减少可用于制糖的蔗糖量；但原糖月度大涨已反映巴西、印度和泰国天气风险，短线继续上冲需要新的供应收缩兑现。来源：Investing.com Brasil/Reuters（https://br.investing.com/news/stock-market-news/acucar-bruto-sobe-na-bolsa-ice-e-fecha-agosto-com-alta-de-215-devido-ao-el-nino-2053623）。影响：利多糖价</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>利多：原糖价格上涨与巴西乙醇回报改善共同指向制糖用蔗减少，若糖厂维持较高乙醇产量，将压缩食糖供应并支撑国际糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="145" customHeight="1" s="2">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>巴西国家供应公司Conab启动东北部独立蔗农经济补贴申请，补贴标准为每吨甘蔗12雷亚尔，项目资金上限2.70亿雷亚尔，覆盖2025/26榨季已商业化的东北部甘蔗。该补贴提高东北部蔗农售蔗收入并帮助维持糖厂原料供应，但区域产量占巴西出口糖供应比例有限，短期难以改变国际食糖供需。来源：Canal da Cana（https://canaldacana.com.br/post-single.php?idnoticia=14487）。影响：中性</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>中性：补贴有助于稳定巴西东北部甘蔗供应，但该区域对巴西出口糖总量影响有限，短期难以改变国际食糖供需。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="180" customHeight="1" s="2">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>印度糖厂公布食糖价格和市场流通，糖价下跌30%。印度食糖价格上涨说明现货供应偏紧或节前需求增强，价格下跌则说明供应压力或需求转弱正在传导到现货端。来源：Business Standard（https://www.business-standard.com/amp/industry/news/ex-mill-sugar-prices-fall-30-pc-but-retail-rates-yet-to-reflect-the-cut-126083100647_1.html）。影响：利空糖价</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>利空：现货或出厂报价下跌反映供应压力或需求转弱，会压制短期糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="162.6" customHeight="1" s="2">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>印度食品和公共分配部将2026年9月上半月国内食糖销售配额定为130万吨，并要求糖厂第一周销售或发运40%；ChiniMandi市场更新显示，马哈拉施特拉S级糖厂价约₹5200-5350/公担、卡纳塔克南部约₹5500/公担、北方邦M/30约₹5050-5100/公担，主要产区报价继续下跌₹100-200/公担。半月配额和首周集中销售要求会增加节前国内可流通糖源，报价回落说明政策投放正在缓解印度现货紧张并压制印度国内糖价。来源：ChiniMandi（https://www.chinimandi.com/daily-sugar-market-update-by-vizzie-31-08-2026/）。影响：利空糖价</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>利空：印度半月销售配额和首周40%销售要求增加国内可流通糖源，糖厂出厂价继续下跌说明政策投放缓解现货紧张，对印度国内糖价形成压力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1" s="2">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>印度政府公布食糖价格和市场流通，糖价或相关政策基准为Rs 60。印度食糖价格上涨说明现货供应偏紧或节前需求增强，价格下跌则说明供应压力或需求转弱正在传导到现货端。来源：The New Indian Express（https://www.newindianexpress.com/india/2026/Aug/30/sugar-prices-stay-above-rs-60kg-in-most-markets-despite-centres-measures-to-curb-rise）。影响：利多糖价</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>利多：现货或出厂报价上涨反映阶段性供应偏紧或采购需求增强，会支撑短期糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="141.7" customHeight="1" s="2">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>印度糖业相关机构公布库存数据，库存增加13%。库存增加会提高现货供应缓冲，压制补库需求和糖价。来源：Business Standard（https://www.business-standard.com/amp/markets/news/sugar-stocks-rebound-balrampur-shree-renuka-triveni-rally-up-to-13-126083100510_1.html）。影响：利空糖价</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>利空：库存增加会提高现货供应缓冲，压制补库需求和糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="140.6" customHeight="1" s="2">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>印度主产区农业或气象机构下调甘蔗产区天气、干旱或病虫害，已说明甘蔗虫害扩散或产区天气风险。印度产区若出现虫害、干旱或洪涝，会压低受影响地块单产并削弱糖料供应稳定性。来源：ChiniMandi（https://www.chinimandi.com/bihar-sugarcane-output-may-decline-amid-lower-acreage-weather-and-pest-concerns/）。影响：利多糖价</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>利多：干旱、洪涝或病虫害会压低甘蔗单产并削弱糖料供应稳定性，从而支撑糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="135.65" customHeight="1" s="2">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>印度政府公布食糖价格和市场流通，糖价下跌30%。印度食糖价格上涨说明现货供应偏紧或节前需求增强，价格下跌则说明供应压力或需求转弱正在传导到现货端。来源：ChiniMandi（https://www.chinimandi.com/ex-mill-sugar-prices-fall-30-after-government-measures-retail-rates-yet-to-ease/）。影响：利空糖价</t>
+          <t>印度气象部门预计9月全国降雨低于正常水平，Reuters报道指出8月降雨已较常年少16%、9月降雨预计低于长期均值的91%，马哈拉施特拉邦和卡纳塔克邦等半岛印度主产区仍处甘蔗生长期。甘蔗生长期降雨不足会削弱田间墒情和单产恢复，若偏少降雨延续到主产区，将降低后期甘蔗供应预期并支撑印度国内糖价。来源：MarketScreener/Reuters（https://www.marketscreener.com/news/india-expects-below-average-september-rains-after-weak-august-ce7858dcd18bff27）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>利空：现货或出厂报价下跌反映供应压力或需求转弱，会压制短期糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="180" customHeight="1" s="2">
+          <t>利多：印度主产区甘蔗生长期降雨偏少会削弱墒情和单产恢复，从而减少后期甘蔗供应预期并支撑印度国内糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="126.3" customHeight="1" s="2">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>印度政府公布食糖价格和市场流通，糖价或相关政策基准为15天。印度食糖价格上涨说明现货供应偏紧或节前需求增强，价格下跌则说明供应压力或需求转弱正在传导到现货端。来源：The Times of India（https://timesofindia.indiatimes.com/city/kolhapur/sugar-cane-crushing-season-may-start-15-days-early-as-maharashtra-govt-moves-to-cool-sugar-prices/amp_articleshow/133636450.cms）。影响：中性</t>
+          <t>泰国气象局预报，东北部、北部、中部及东部甘蔗产区在8月31日至9月1日前后仍有雷阵雨和局地大雨，涉及乌隆他尼、孔敬、呵叻、加拉信、黎府、甘烹碧、彭世洛、北碧和沙缴等主产区。泰国甘蔗处于生长期，雷阵雨和局地大雨补充土壤水分并改善墒情，有利于单产形成和后期食糖产量恢复。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>中性：价格信息缺少明确涨跌幅或区域基准，暂不改变供需判断。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="137.3" customHeight="1" s="2">
+          <t>利空：泰国主产区生长期降雨会补充土壤水分、改善墒情并促进甘蔗单产形成，从而增加后期甘蔗和食糖供应预期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="153.25" customHeight="1" s="2">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>中国</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构发布或调整食糖贸易、进口、出口或配额政策，贸易政策数量为130万吨。进口放宽会补充进口国国内糖源并压制本地现货；出口配额增加会提高国际可流通糖源，出口限制则减少国际供应。来源：ChiniMandi（https://www.chinimandi.com/13-lmt-sugar-quota-fixed-for-first-fortnight-of-september-2026/）。影响：利多糖价</t>
+          <t>第19号台风“紫檀”引发洪涝，广西宁明县海渊镇10.3万亩甘蔗中有2.5万亩受灾，海渊镇和广西海棠东亚糖业有限公司通过遥感、无人机和实地核查受灾地块并开展排涝扶苗。受淹、倒伏和长时间积水会削弱受灾蔗区单产，若绝收地块扩大，将减少广西新榨季可供糖厂压榨的甘蔗量，对国内糖价形成支撑。来源：泛糖科技/宁明县融媒体中心（https://www.hisugar.com/home/articleContent?id=2026083113575898619866）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>利多：出口限制、配额收紧或贸易成本上升会减少可流通糖源并支撑国际糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="180" customHeight="1" s="2">
+          <t>利多：广西甘蔗受淹和倒伏会降低受灾蔗区单产并减少新榨季糖厂原料供应，从而支撑国内糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="171.95" customHeight="1" s="2">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>中国</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Open-Meteo预报显示（2026-09-01至2026-09-07），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括乌隆他尼约130.7mm、黎府约116.1mm、加拉信约115.6mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
+          <t>泛糖科技国内制糖集团报价显示，广西白糖现货主流成交价为5121元/吨，较前一日下跌30元/吨；南华广西一级糖报价5170-5230元/吨、下调20元/吨，云南南华昆明报价5050元/吨、祥云和大理5010元/吨、下调10元/吨。广西和云南现货报价下调说明终端采购节奏放缓，短线对国内现货糖价形成压力；但台风后广西蔗区受灾限制新榨季原料预期，价格下跌对供需判断的影响有限。来源：泛糖科技（https://www.hisugar.com/home/articleContent?id=2026083116065411487699）。影响：中性</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="146.65" customHeight="1" s="2">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>南非</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>南非糖业相关机构提高食糖贸易、进口、出口或配额政策，贸易政策披露$785。进口放宽会补充进口国国内糖源并压制本地现货；出口配额增加会提高国际可流通糖源，出口限制则减少国际供应。来源：ChiniMandi（https://www.chinimandi.com/south-africa-raises-sugar-import-benchmark-to-785-industry-seeks-stronger-protection/）。影响：利空糖价</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>利空：进口政策放宽或进口量增加会补充国内可用糖源，对本地糖价形成压力。</t>
+          <t>中性：广西和云南报价下调会压制短线现货糖价，但灾后原料供应风险仍在，国内糖价暂未形成明确单边供需信号。</t>
         </is>
       </c>
     </row>

</xml_diff>